<commit_message>
Atualizando base de dados com as novas coordenadas para a apresentacao
</commit_message>
<xml_diff>
--- a/Transporte Gestores (1).xlsx
+++ b/Transporte Gestores (1).xlsx
@@ -7320,7 +7320,7 @@
     <row r="30">
       <c r="B30" s="51" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Mikaella Ribeiro Molina  </t>
+          <t>Mikaella Ribeiro Molina</t>
         </is>
       </c>
       <c r="C30" s="51" t="inlineStr">
@@ -7341,13 +7341,23 @@
       <c r="F30" s="51" t="inlineStr">
         <is>
           <t>64 99237-9738</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>-18.422867739570577</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>-49.24333547153385</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="B31" s="51" t="inlineStr">
         <is>
-          <t xml:space="preserve">Grazielle Btista da Silva Dafico Ramos </t>
+          <t>Grazielle Btista da Silva Dafico Ramos</t>
         </is>
       </c>
       <c r="C31" s="51" t="inlineStr">
@@ -7368,6 +7378,16 @@
       <c r="F31" s="51" t="inlineStr">
         <is>
           <t>62 98214-1634</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>-18.4308187104198</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>-49.216809289244246</t>
         </is>
       </c>
     </row>
@@ -7397,6 +7417,16 @@
           <t>64 9999-5660</t>
         </is>
       </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>-18.417045561657343</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>-49.220856886291514</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="B33" s="51" t="inlineStr">
@@ -7424,6 +7454,16 @@
           <t>64 99324-8939</t>
         </is>
       </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>-18.40306479197539</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>-49.21985746510261</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="B34" s="51" t="inlineStr">
@@ -7451,6 +7491,16 @@
           <t>64 99201-4066</t>
         </is>
       </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>-18.390932153882023</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>-49.200576690191276</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="B35" s="51" t="inlineStr">
@@ -7478,6 +7528,16 @@
           <t>64 99297-8715</t>
         </is>
       </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>-18.37893736807591</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>-49.21423266310902</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="B36" s="51" t="inlineStr">
@@ -7498,6 +7558,16 @@
       <c r="F36" s="51" t="inlineStr">
         <is>
           <t>64 99289-9736</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>-18.388358425785132</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>-49.213702522758524</t>
         </is>
       </c>
     </row>

</xml_diff>